<commit_message>
Preserve local vacancy analysis changes
</commit_message>
<xml_diff>
--- a/analysis/vacancy_v_sdes.xlsx
+++ b/analysis/vacancy_v_sdes.xlsx
@@ -76,12 +76,12 @@
     <t>T</t>
   </si>
   <si>
+    <t>D</t>
+  </si>
+  <si>
     <t>E</t>
   </si>
   <si>
-    <t>D</t>
-  </si>
-  <si>
     <t>labels_full</t>
   </si>
   <si>
@@ -142,12 +142,12 @@
     <t>T - Activities of households as employers; undifferentiated goods- and services-producing activities of households for own use</t>
   </si>
   <si>
+    <t>D - Electricity, gas, steam and air conditioning supply</t>
+  </si>
+  <si>
     <t>E - Water supply; sewerage, waste management and remediation activities</t>
   </si>
   <si>
-    <t>D - Electricity, gas, steam and air conditioning supply</t>
-  </si>
-  <si>
     <t>label_short</t>
   </si>
   <si>
@@ -208,10 +208,10 @@
     <t>Activities of households as employers</t>
   </si>
   <si>
+    <t>Electricity, gas, steam and air conditioning supply</t>
+  </si>
+  <si>
     <t>Water supply, sewerage, waste management</t>
-  </si>
-  <si>
-    <t>Electricity, gas, steam and air conditioning supply</t>
   </si>
   <si>
     <t>sdes_share</t>
@@ -677,7 +677,7 @@
         <v>64</v>
       </c>
       <c r="D21" s="0">
-        <v>0.0003816229582298547</v>
+        <v>0.0014760036719962955</v>
       </c>
       <c r="E21" s="0">
         <v>0</v>
@@ -694,7 +694,7 @@
         <v>65</v>
       </c>
       <c r="D22" s="0">
-        <v>0.0014760036719962955</v>
+        <v>0.0003816229582298547</v>
       </c>
       <c r="E22" s="0">
         <v>0</v>

</xml_diff>